<commit_message>
docs(rfp): cut the vendor email to essentials; stop coaching how to answer
These vendors know the industry. Defining capacity and scheduling for them
reads as filler, and the supplementary material covers it. The email now says
who we are, what we are looking at, the date, and the timeline.

States that we are home health and hospice, currently focused on the home
health side, with an interest in carrying it over to hospice later.

Removes every instruction on how to answer — from the email and from the
workbook Instructions tab, which carried the same guidance. Let them answer the
way they are going to answer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UvRGJ3Qj1APfQLfybFmnqq
</commit_message>
<xml_diff>
--- a/agents/compassus-capacity-pm/rfp/Compassus-Vendor-Questionnaire-MASTER.xlsx
+++ b/agents/compassus-capacity-pm/rfp/Compassus-Vendor-Questionnaire-MASTER.xlsx
@@ -862,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E22"/>
+  <dimension ref="B2:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -904,95 +904,79 @@
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Answering</t>
+          <t>Practical notes</t>
         </is>
       </c>
     </row>
     <row r="9" ht="35" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Answer in your own words. Most answers run a short paragraph. There is no advantage in volume, and where something does not apply to your product, saying so plainly is a genuinely useful answer.</t>
+          <t>Press Alt+Enter to start a new paragraph inside a cell. Press Ctrl+Shift+U to expand the formula bar if you would rather write there. You can drag any row taller if you need more room.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Practical notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="35" customHeight="1">
+          <t>Working as a team</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Press Alt+Enter to start a new paragraph inside a cell. Press Ctrl+Shift+U to expand the formula bar if you would rather write there. You can drag any row taller if you need more room — the height we set is only a suggestion of length.</t>
+          <t>If several people need to contribute, put the file in your own SharePoint or Drive to co-author it, then send the completed workbook back.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Working as a team</t>
+          <t>The Overview tab</t>
         </is>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>If several people need to contribute, put the file in your own SharePoint or Drive to co-author it, then send the completed workbook back.</t>
+          <t>The Overview tab reproduces the one-page summary of what we are looking for. It is there for reference while you answer.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>The Overview tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="21" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>The Overview tab reproduces the one-page summary of what we are looking for. It is there for reference while you answer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
           <t>Progress</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="5">
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="5">
         <f>COUNTA(Questionnaire!E9,Questionnaire!E11,Questionnaire!E13,Questionnaire!E15,Questionnaire!E37,Questionnaire!E39,Questionnaire!E41,Questionnaire!E43,Questionnaire!E45,Questionnaire!E47,Questionnaire!E53,Questionnaire!E55,Questionnaire!E57,Questionnaire!E59,Questionnaire!E64,Questionnaire!E66,Questionnaire!E68) &amp; " of 17 questions answered"</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="6" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Updates as you type. Counts the answer cells only, not the coverage grid.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B20:E20"/>
+  <mergeCells count="13">
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B19:E19"/>
     <mergeCell ref="B14:E14"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>